<commit_message>
feat: update FIXED and WK36 excel templates
</commit_message>
<xml_diff>
--- a/Dashboard_Template_30_Slides_Final_WK36.xlsx
+++ b/Dashboard_Template_30_Slides_Final_WK36.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0_Agent\0_Dashboad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A41ABB49-BE5B-478D-9E53-C74520C7AFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3BA476-F721-45CB-A568-052FA65BAECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="748" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="Part 4 - Financials" sheetId="4" r:id="rId4"/>
     <sheet name="Part 5 - Safety" sheetId="5" r:id="rId5"/>
     <sheet name="Part 7 - SLA On-Process TRUE" sheetId="6" r:id="rId6"/>
-    <sheet name="Part 7 - SLA On-Process" sheetId="7" r:id="rId7"/>
+    <sheet name="Part 7 - SLA On-Process AIS" sheetId="7" r:id="rId7"/>
     <sheet name="2026" sheetId="8" r:id="rId8"/>
     <sheet name="Sheet1" sheetId="9" r:id="rId9"/>
   </sheets>

</xml_diff>